<commit_message>
Update system to automatically save patient data to Excel
Modify the autosave functionality in main.py to also write patient data to hospital_patients.xlsx in addition to hospital_patients.csv.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c752e2c9-3044-42a3-b331-4756feaa10ab
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,6 +483,34 @@
         <v>8</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>age &gt; 20 and score &gt; 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>erris</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ehadache</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>age &gt; 20 and score &gt; 8</t>
         </is>

</xml_diff>

<commit_message>
Add ability to export patient data to an Excel file
Append patient data to the 'hospital_patients.xlsx' file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b381ff69-37d5-45b0-837b-abe871dcb9d8
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,34 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>age &gt; 20 and score &gt; 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>rrona</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>age &gt; 21 and score &gt; 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update patient data management to manual save and load operations
Removed automatic CSV and Excel saving/exporting, simplifying file operations to manual "Save to CSV" and "Load from CSV" actions.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4230396a-aab0-45c7-b807-ec5fd97d594c
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,6 +543,30 @@
           <t>age &gt; 21 and score &gt; 9</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>erris</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>covid</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Automatically save patient data to both CSV and Excel files
Update the auto-save functionality to write patient data to both `hospital_patients.csv` and `hospital_patients.xlsx` when patients are added or edited.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 3d129e40-643d-49c1-ac30-ac00130763a5
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,7 +566,151 @@
       <c r="E5" t="n">
         <v>10</v>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1111</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>erris</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>23</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>age &gt; 23 and score &gt; 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P999</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>age &gt; 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>erris</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>hh</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>age &gt; 25 and score &gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>erris</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>age &gt; 22 and score &gt; 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>28</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Asthma</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>age &gt; 25</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add functionality to delete patients and update files
Adds a new menu option to delete patients by ID, and updates the autosave functionality to include deleting from both CSV and Excel files.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5c97db91-156a-4f17-9ca3-f26480b8ce9c
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -687,28 +687,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>999999</t>
+          <t>333</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sarah</t>
+          <t>erris</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Asthma</t>
+          <t>qq</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>age &gt; 25</t>
+          <t>nan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a truth table display and performance comparison for sorting algorithms
Implement an abstract base class for sorting strategies, add a truth table display method, and create a performance comparison feature for sorting algorithms.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 05fa91ab-c578-4acc-9827-c5a9d1ef5e02
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,237 +480,9 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>age &gt; 20 and score &gt; 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>erris</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ehadache</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>age &gt; 20 and score &gt; 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>rrona</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>21</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
         <v>9</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>age &gt; 21 and score &gt; 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>erris</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>20</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>covid</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1111</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>erris</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>23</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>age &gt; 23 and score &gt; 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>P999</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Test User</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Fever</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>age &gt; 25</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1234</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>erris</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>25</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>hh</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>age &gt; 25 and score &gt; 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>erris</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>22</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>age &gt; 22 and score &gt; 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>333</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>erris</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>11</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>qq</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add a detailed patient report with risk and age classifications
Introduce PatientReport as a subclass of Patient, adding attributes for risk level, age group, and notes. Includes methods to classify risk and age, and overrides to_tuple and adds a summary method.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 69d84769-8295-4125-8957-aabeb00b5519
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 34ab3122-1c6c-4fd5-9fad-30cbfe0ae290
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/hospital_patients.xlsx
+++ b/hospital_patients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,7 +482,39 @@
       <c r="E2" t="n">
         <v>9</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>erris</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>age 21 &gt; and scorre &gt; 9</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>